<commit_message>
updated AVCMDS worksheet template (replaced stray company-specific language with generic)
</commit_message>
<xml_diff>
--- a/distribution/reference_documents/templates/AVCMDS Worksheet template.xlsx
+++ b/distribution/reference_documents/templates/AVCMDS Worksheet template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charles.wilson/Documents/projects/AVCDL/source/reference_documents/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA1233B-3061-BC4A-A505-317AB1F1BB1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED0FF3D3-9A69-A042-898F-21964E680AEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19100" yWindow="3420" windowWidth="21760" windowHeight="36860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30060" yWindow="2380" windowWidth="21760" windowHeight="36860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AVCMDS form" sheetId="1" r:id="rId1"/>
@@ -580,9 +580,6 @@
   </si>
   <si>
     <t>AUTH-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Can the device manufacturer or Motional grant themselves unrestricted administrative privileges (e.g., access operating system or application via local root or administrator account)?  </t>
   </si>
   <si>
     <t>AUTH-4</t>
@@ -1976,6 +1973,9 @@
   </si>
   <si>
     <t>Rev 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can the device manufacturer or other entity grant themselves unrestricted administrative privileges (e.g., access operating system or application via local root or administrator account)?  </t>
   </si>
 </sst>
 </file>
@@ -2333,8 +2333,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2342,28 +2342,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2373,7 +2352,28 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2608,17 +2608,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="24" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
-        <v>628</v>
-      </c>
-      <c r="B1" s="53"/>
-      <c r="C1" s="53"/>
-      <c r="D1" s="53"/>
+      <c r="A1" s="43" t="s">
+        <v>627</v>
+      </c>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="2" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
@@ -2639,10 +2639,10 @@
       <c r="Y1" s="3"/>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A2" s="54"/>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
+      <c r="A2" s="45"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
@@ -2693,7 +2693,7 @@
       </c>
     </row>
     <row r="5" spans="1:25" ht="19" x14ac:dyDescent="0.25">
-      <c r="A5" s="56"/>
+      <c r="A5" s="48"/>
       <c r="B5" s="39"/>
       <c r="C5" s="39"/>
       <c r="D5" s="39"/>
@@ -2763,7 +2763,7 @@
       <c r="Y6" s="10"/>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A7" s="55"/>
+      <c r="A7" s="46"/>
       <c r="B7" s="39"/>
       <c r="C7" s="39"/>
       <c r="D7" s="39"/>
@@ -3025,7 +3025,7 @@
       <c r="H23" s="19"/>
     </row>
     <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="48"/>
+      <c r="A24" s="47"/>
       <c r="B24" s="39"/>
       <c r="C24" s="39"/>
       <c r="D24" s="39"/>
@@ -3196,7 +3196,7 @@
         <v>69</v>
       </c>
       <c r="B33" s="34" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="C33" s="22" t="s">
         <v>54</v>
@@ -3480,7 +3480,7 @@
       <c r="H47" s="19"/>
     </row>
     <row r="48" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="48"/>
+      <c r="A48" s="47"/>
       <c r="B48" s="39"/>
       <c r="C48" s="39"/>
       <c r="D48" s="39"/>
@@ -3519,7 +3519,7 @@
       <c r="Y49" s="23"/>
     </row>
     <row r="50" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="47" t="s">
+      <c r="A50" s="38" t="s">
         <v>99</v>
       </c>
       <c r="B50" s="39"/>
@@ -3547,7 +3547,7 @@
       <c r="H51" s="19"/>
     </row>
     <row r="52" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="38"/>
+      <c r="A52" s="42"/>
       <c r="B52" s="39"/>
       <c r="C52" s="39"/>
       <c r="D52" s="39"/>
@@ -3569,7 +3569,7 @@
       <c r="H53" s="40"/>
     </row>
     <row r="54" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="47" t="s">
+      <c r="A54" s="38" t="s">
         <v>103</v>
       </c>
       <c r="B54" s="39"/>
@@ -3645,7 +3645,7 @@
         <v>115</v>
       </c>
       <c r="B58" s="34" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="C58" s="22" t="s">
         <v>35</v>
@@ -4221,7 +4221,7 @@
       <c r="H86" s="19"/>
     </row>
     <row r="87" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A87" s="38"/>
+      <c r="A87" s="42"/>
       <c r="B87" s="39"/>
       <c r="C87" s="39"/>
       <c r="D87" s="39"/>
@@ -4243,7 +4243,7 @@
       <c r="H88" s="40"/>
     </row>
     <row r="89" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A89" s="47" t="s">
+      <c r="A89" s="38" t="s">
         <v>173</v>
       </c>
       <c r="B89" s="39"/>
@@ -4302,8 +4302,8 @@
       <c r="A92" s="25" t="s">
         <v>181</v>
       </c>
-      <c r="B92" s="16" t="s">
-        <v>182</v>
+      <c r="B92" s="34" t="s">
+        <v>631</v>
       </c>
       <c r="C92" s="22" t="s">
         <v>54</v>
@@ -4322,10 +4322,10 @@
     </row>
     <row r="93" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="25" t="s">
+        <v>182</v>
+      </c>
+      <c r="B93" s="16" t="s">
         <v>183</v>
-      </c>
-      <c r="B93" s="16" t="s">
-        <v>184</v>
       </c>
       <c r="C93" s="22" t="s">
         <v>44</v>
@@ -4344,10 +4344,10 @@
     </row>
     <row r="94" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="25" t="s">
+        <v>184</v>
+      </c>
+      <c r="B94" s="16" t="s">
         <v>185</v>
-      </c>
-      <c r="B94" s="16" t="s">
-        <v>186</v>
       </c>
       <c r="C94" s="22" t="s">
         <v>44</v>
@@ -4359,7 +4359,7 @@
       <c r="H94" s="19"/>
     </row>
     <row r="95" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A95" s="38"/>
+      <c r="A95" s="42"/>
       <c r="B95" s="39"/>
       <c r="C95" s="39"/>
       <c r="D95" s="39"/>
@@ -4370,7 +4370,7 @@
     </row>
     <row r="96" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="41" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B96" s="39"/>
       <c r="C96" s="39"/>
@@ -4381,8 +4381,8 @@
       <c r="H96" s="40"/>
     </row>
     <row r="97" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="47" t="s">
-        <v>188</v>
+      <c r="A97" s="38" t="s">
+        <v>187</v>
       </c>
       <c r="B97" s="39"/>
       <c r="C97" s="39"/>
@@ -4394,10 +4394,10 @@
     </row>
     <row r="98" spans="1:8" ht="64" x14ac:dyDescent="0.2">
       <c r="A98" s="25" t="s">
+        <v>188</v>
+      </c>
+      <c r="B98" s="16" t="s">
         <v>189</v>
-      </c>
-      <c r="B98" s="16" t="s">
-        <v>190</v>
       </c>
       <c r="C98" s="22" t="s">
         <v>44</v>
@@ -4410,10 +4410,10 @@
     </row>
     <row r="99" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="25" t="s">
+        <v>190</v>
+      </c>
+      <c r="B99" s="16" t="s">
         <v>191</v>
-      </c>
-      <c r="B99" s="16" t="s">
-        <v>192</v>
       </c>
       <c r="C99" s="22" t="s">
         <v>44</v>
@@ -4426,10 +4426,10 @@
     </row>
     <row r="100" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A100" s="25" t="s">
+        <v>192</v>
+      </c>
+      <c r="B100" s="16" t="s">
         <v>193</v>
-      </c>
-      <c r="B100" s="16" t="s">
-        <v>194</v>
       </c>
       <c r="C100" s="22" t="s">
         <v>44</v>
@@ -4442,10 +4442,10 @@
     </row>
     <row r="101" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A101" s="25" t="s">
+        <v>194</v>
+      </c>
+      <c r="B101" s="16" t="s">
         <v>195</v>
-      </c>
-      <c r="B101" s="16" t="s">
-        <v>196</v>
       </c>
       <c r="C101" s="22" t="s">
         <v>44</v>
@@ -4458,10 +4458,10 @@
     </row>
     <row r="102" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A102" s="25" t="s">
+        <v>196</v>
+      </c>
+      <c r="B102" s="16" t="s">
         <v>197</v>
-      </c>
-      <c r="B102" s="16" t="s">
-        <v>198</v>
       </c>
       <c r="C102" s="22" t="s">
         <v>44</v>
@@ -4474,10 +4474,10 @@
     </row>
     <row r="103" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A103" s="25" t="s">
+        <v>198</v>
+      </c>
+      <c r="B103" s="16" t="s">
         <v>199</v>
-      </c>
-      <c r="B103" s="16" t="s">
-        <v>200</v>
       </c>
       <c r="C103" s="22" t="s">
         <v>44</v>
@@ -4490,10 +4490,10 @@
     </row>
     <row r="104" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A104" s="25" t="s">
+        <v>200</v>
+      </c>
+      <c r="B104" s="16" t="s">
         <v>201</v>
-      </c>
-      <c r="B104" s="16" t="s">
-        <v>202</v>
       </c>
       <c r="C104" s="22" t="s">
         <v>44</v>
@@ -4506,10 +4506,10 @@
     </row>
     <row r="105" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A105" s="25" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B105" s="16" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C105" s="22" t="s">
         <v>44</v>
@@ -4522,10 +4522,10 @@
     </row>
     <row r="106" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A106" s="25" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B106" s="16" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C106" s="22" t="s">
         <v>44</v>
@@ -4538,10 +4538,10 @@
     </row>
     <row r="107" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A107" s="25" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B107" s="16" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C107" s="22" t="s">
         <v>44</v>
@@ -4554,10 +4554,10 @@
     </row>
     <row r="108" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A108" s="25" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B108" s="16" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C108" s="22" t="s">
         <v>35</v>
@@ -4570,10 +4570,10 @@
     </row>
     <row r="109" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A109" s="25" t="s">
+        <v>206</v>
+      </c>
+      <c r="B109" s="16" t="s">
         <v>207</v>
-      </c>
-      <c r="B109" s="16" t="s">
-        <v>208</v>
       </c>
       <c r="C109" s="22" t="s">
         <v>44</v>
@@ -4586,10 +4586,10 @@
     </row>
     <row r="110" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A110" s="25" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B110" s="16" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C110" s="22" t="s">
         <v>44</v>
@@ -4602,10 +4602,10 @@
     </row>
     <row r="111" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A111" s="25" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B111" s="16" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C111" s="22" t="s">
         <v>44</v>
@@ -4618,10 +4618,10 @@
     </row>
     <row r="112" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A112" s="25" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B112" s="16" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C112" s="22" t="s">
         <v>44</v>
@@ -4634,10 +4634,10 @@
     </row>
     <row r="113" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A113" s="25" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B113" s="16" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C113" s="22" t="s">
         <v>44</v>
@@ -4650,10 +4650,10 @@
     </row>
     <row r="114" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="25" t="s">
+        <v>212</v>
+      </c>
+      <c r="B114" s="16" t="s">
         <v>213</v>
-      </c>
-      <c r="B114" s="16" t="s">
-        <v>214</v>
       </c>
       <c r="C114" s="22" t="s">
         <v>44</v>
@@ -4666,10 +4666,10 @@
     </row>
     <row r="115" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A115" s="25" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B115" s="16" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C115" s="22" t="s">
         <v>44</v>
@@ -4682,10 +4682,10 @@
     </row>
     <row r="116" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A116" s="25" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B116" s="16" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C116" s="22" t="s">
         <v>44</v>
@@ -4698,10 +4698,10 @@
     </row>
     <row r="117" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A117" s="25" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B117" s="16" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C117" s="22" t="s">
         <v>44</v>
@@ -4714,10 +4714,10 @@
     </row>
     <row r="118" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A118" s="25" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B118" s="16" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C118" s="22" t="s">
         <v>44</v>
@@ -4730,10 +4730,10 @@
     </row>
     <row r="119" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A119" s="25" t="s">
+        <v>218</v>
+      </c>
+      <c r="B119" s="16" t="s">
         <v>219</v>
-      </c>
-      <c r="B119" s="16" t="s">
-        <v>220</v>
       </c>
       <c r="C119" s="22" t="s">
         <v>44</v>
@@ -4746,10 +4746,10 @@
     </row>
     <row r="120" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A120" s="25" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B120" s="16" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C120" s="22" t="s">
         <v>44</v>
@@ -4762,10 +4762,10 @@
     </row>
     <row r="121" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A121" s="25" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B121" s="16" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C121" s="22" t="s">
         <v>44</v>
@@ -4778,10 +4778,10 @@
     </row>
     <row r="122" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A122" s="25" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B122" s="16" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C122" s="22" t="s">
         <v>44</v>
@@ -4794,10 +4794,10 @@
     </row>
     <row r="123" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A123" s="25" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B123" s="16" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C123" s="22" t="s">
         <v>44</v>
@@ -4810,10 +4810,10 @@
     </row>
     <row r="124" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A124" s="25" t="s">
+        <v>224</v>
+      </c>
+      <c r="B124" s="16" t="s">
         <v>225</v>
-      </c>
-      <c r="B124" s="16" t="s">
-        <v>226</v>
       </c>
       <c r="C124" s="22" t="s">
         <v>44</v>
@@ -4826,10 +4826,10 @@
     </row>
     <row r="125" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="25" t="s">
+        <v>226</v>
+      </c>
+      <c r="B125" s="16" t="s">
         <v>227</v>
-      </c>
-      <c r="B125" s="16" t="s">
-        <v>228</v>
       </c>
       <c r="C125" s="22" t="s">
         <v>44</v>
@@ -4842,10 +4842,10 @@
     </row>
     <row r="126" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A126" s="25" t="s">
+        <v>228</v>
+      </c>
+      <c r="B126" s="16" t="s">
         <v>229</v>
-      </c>
-      <c r="B126" s="16" t="s">
-        <v>230</v>
       </c>
       <c r="C126" s="22" t="s">
         <v>44</v>
@@ -4858,10 +4858,10 @@
     </row>
     <row r="127" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A127" s="25" t="s">
+        <v>230</v>
+      </c>
+      <c r="B127" s="16" t="s">
         <v>231</v>
-      </c>
-      <c r="B127" s="16" t="s">
-        <v>232</v>
       </c>
       <c r="C127" s="22" t="s">
         <v>44</v>
@@ -4874,10 +4874,10 @@
     </row>
     <row r="128" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A128" s="25" t="s">
+        <v>232</v>
+      </c>
+      <c r="B128" s="16" t="s">
         <v>233</v>
-      </c>
-      <c r="B128" s="16" t="s">
-        <v>234</v>
       </c>
       <c r="C128" s="22" t="s">
         <v>44</v>
@@ -4890,10 +4890,10 @@
     </row>
     <row r="129" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A129" s="25" t="s">
+        <v>234</v>
+      </c>
+      <c r="B129" s="16" t="s">
         <v>235</v>
-      </c>
-      <c r="B129" s="16" t="s">
-        <v>236</v>
       </c>
       <c r="C129" s="22" t="s">
         <v>35</v>
@@ -4906,10 +4906,10 @@
     </row>
     <row r="130" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="25" t="s">
+        <v>236</v>
+      </c>
+      <c r="B130" s="16" t="s">
         <v>237</v>
-      </c>
-      <c r="B130" s="16" t="s">
-        <v>238</v>
       </c>
       <c r="C130" s="22" t="s">
         <v>44</v>
@@ -4922,10 +4922,10 @@
     </row>
     <row r="131" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="25" t="s">
+        <v>238</v>
+      </c>
+      <c r="B131" s="16" t="s">
         <v>239</v>
-      </c>
-      <c r="B131" s="16" t="s">
-        <v>240</v>
       </c>
       <c r="C131" s="22" t="s">
         <v>44</v>
@@ -4948,7 +4948,7 @@
     </row>
     <row r="133" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="41" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B133" s="39"/>
       <c r="C133" s="39"/>
@@ -4959,8 +4959,8 @@
       <c r="H133" s="40"/>
     </row>
     <row r="134" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A134" s="47" t="s">
-        <v>242</v>
+      <c r="A134" s="38" t="s">
+        <v>241</v>
       </c>
       <c r="B134" s="39"/>
       <c r="C134" s="39"/>
@@ -4972,28 +4972,28 @@
     </row>
     <row r="135" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A135" s="25" t="s">
+        <v>242</v>
+      </c>
+      <c r="B135" s="16" t="s">
         <v>243</v>
-      </c>
-      <c r="B135" s="16" t="s">
-        <v>244</v>
       </c>
       <c r="C135" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D135" s="18"/>
       <c r="E135" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F135" s="4" t="s">
         <v>114</v>
       </c>
       <c r="G135" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="H135" s="19"/>
     </row>
     <row r="136" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A136" s="38"/>
+      <c r="A136" s="42"/>
       <c r="B136" s="39"/>
       <c r="C136" s="39"/>
       <c r="D136" s="39"/>
@@ -5004,7 +5004,7 @@
     </row>
     <row r="137" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="41" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B137" s="39"/>
       <c r="C137" s="39"/>
@@ -5015,8 +5015,8 @@
       <c r="H137" s="40"/>
     </row>
     <row r="138" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A138" s="47" t="s">
-        <v>248</v>
+      <c r="A138" s="38" t="s">
+        <v>247</v>
       </c>
       <c r="B138" s="39"/>
       <c r="C138" s="39"/>
@@ -5028,10 +5028,10 @@
     </row>
     <row r="139" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A139" s="15" t="s">
+        <v>248</v>
+      </c>
+      <c r="B139" s="16" t="s">
         <v>249</v>
-      </c>
-      <c r="B139" s="16" t="s">
-        <v>250</v>
       </c>
       <c r="C139" s="22" t="s">
         <v>35</v>
@@ -5044,32 +5044,32 @@
     </row>
     <row r="140" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A140" s="25" t="s">
+        <v>250</v>
+      </c>
+      <c r="B140" s="16" t="s">
         <v>251</v>
-      </c>
-      <c r="B140" s="16" t="s">
-        <v>252</v>
       </c>
       <c r="C140" s="22" t="s">
         <v>54</v>
       </c>
       <c r="D140" s="18"/>
       <c r="E140" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="F140" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="F140" s="4" t="s">
+      <c r="G140" s="4" t="s">
         <v>254</v>
-      </c>
-      <c r="G140" s="4" t="s">
-        <v>255</v>
       </c>
       <c r="H140" s="19"/>
     </row>
     <row r="141" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="15" t="s">
+        <v>255</v>
+      </c>
+      <c r="B141" s="16" t="s">
         <v>256</v>
-      </c>
-      <c r="B141" s="16" t="s">
-        <v>257</v>
       </c>
       <c r="C141" s="22" t="s">
         <v>35</v>
@@ -5082,32 +5082,32 @@
     </row>
     <row r="142" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="25" t="s">
+        <v>257</v>
+      </c>
+      <c r="B142" s="16" t="s">
         <v>258</v>
-      </c>
-      <c r="B142" s="16" t="s">
-        <v>259</v>
       </c>
       <c r="C142" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D142" s="18"/>
       <c r="E142" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="F142" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="F142" s="4" t="s">
+      <c r="G142" s="4" t="s">
         <v>254</v>
-      </c>
-      <c r="G142" s="4" t="s">
-        <v>255</v>
       </c>
       <c r="H142" s="19"/>
     </row>
     <row r="143" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="25" t="s">
+        <v>259</v>
+      </c>
+      <c r="B143" s="16" t="s">
         <v>260</v>
-      </c>
-      <c r="B143" s="16" t="s">
-        <v>261</v>
       </c>
       <c r="C143" s="22" t="s">
         <v>35</v>
@@ -5120,10 +5120,10 @@
     </row>
     <row r="144" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A144" s="25" t="s">
+        <v>261</v>
+      </c>
+      <c r="B144" s="16" t="s">
         <v>262</v>
-      </c>
-      <c r="B144" s="16" t="s">
-        <v>263</v>
       </c>
       <c r="C144" s="22" t="s">
         <v>54</v>
@@ -5136,28 +5136,28 @@
     </row>
     <row r="145" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A145" s="25" t="s">
+        <v>263</v>
+      </c>
+      <c r="B145" s="16" t="s">
         <v>264</v>
-      </c>
-      <c r="B145" s="16" t="s">
-        <v>265</v>
       </c>
       <c r="C145" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D145" s="18"/>
       <c r="E145" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="F145" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="F145" s="4" t="s">
+      <c r="G145" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="G145" s="4" t="s">
-        <v>255</v>
-      </c>
       <c r="H145" s="19"/>
     </row>
     <row r="146" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A146" s="38"/>
+      <c r="A146" s="42"/>
       <c r="B146" s="39"/>
       <c r="C146" s="39"/>
       <c r="D146" s="39"/>
@@ -5168,7 +5168,7 @@
     </row>
     <row r="147" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="41" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B147" s="39"/>
       <c r="C147" s="39"/>
@@ -5179,8 +5179,8 @@
       <c r="H147" s="40"/>
     </row>
     <row r="148" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A148" s="47" t="s">
-        <v>267</v>
+      <c r="A148" s="38" t="s">
+        <v>266</v>
       </c>
       <c r="B148" s="39"/>
       <c r="C148" s="39"/>
@@ -5192,50 +5192,50 @@
     </row>
     <row r="149" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A149" s="25" t="s">
+        <v>267</v>
+      </c>
+      <c r="B149" s="16" t="s">
         <v>268</v>
-      </c>
-      <c r="B149" s="16" t="s">
-        <v>269</v>
       </c>
       <c r="C149" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D149" s="18"/>
       <c r="E149" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="F149" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="F149" s="4" t="s">
+      <c r="G149" s="4" t="s">
         <v>271</v>
-      </c>
-      <c r="G149" s="4" t="s">
-        <v>272</v>
       </c>
       <c r="H149" s="19"/>
     </row>
     <row r="150" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A150" s="25" t="s">
+        <v>272</v>
+      </c>
+      <c r="B150" s="16" t="s">
         <v>273</v>
-      </c>
-      <c r="B150" s="16" t="s">
-        <v>274</v>
       </c>
       <c r="C150" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D150" s="18"/>
       <c r="E150" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="F150" s="4" t="s">
         <v>270</v>
       </c>
-      <c r="F150" s="4" t="s">
+      <c r="G150" s="4" t="s">
         <v>271</v>
       </c>
-      <c r="G150" s="4" t="s">
-        <v>272</v>
-      </c>
       <c r="H150" s="19"/>
     </row>
     <row r="151" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A151" s="38"/>
+      <c r="A151" s="42"/>
       <c r="B151" s="39"/>
       <c r="C151" s="39"/>
       <c r="D151" s="39"/>
@@ -5246,7 +5246,7 @@
     </row>
     <row r="152" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="41" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B152" s="39"/>
       <c r="C152" s="39"/>
@@ -5257,8 +5257,8 @@
       <c r="H152" s="40"/>
     </row>
     <row r="153" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A153" s="47" t="s">
-        <v>276</v>
+      <c r="A153" s="38" t="s">
+        <v>275</v>
       </c>
       <c r="B153" s="39"/>
       <c r="C153" s="39"/>
@@ -5270,19 +5270,19 @@
     </row>
     <row r="154" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="25" t="s">
+        <v>276</v>
+      </c>
+      <c r="B154" s="16" t="s">
         <v>277</v>
-      </c>
-      <c r="B154" s="16" t="s">
-        <v>278</v>
       </c>
       <c r="C154" s="22" t="s">
         <v>54</v>
       </c>
       <c r="D154" s="24" t="s">
+        <v>278</v>
+      </c>
+      <c r="E154" s="4" t="s">
         <v>279</v>
-      </c>
-      <c r="E154" s="4" t="s">
-        <v>280</v>
       </c>
       <c r="F154" s="4"/>
       <c r="G154" s="4"/>
@@ -5290,105 +5290,105 @@
     </row>
     <row r="155" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A155" s="25" t="s">
+        <v>280</v>
+      </c>
+      <c r="B155" s="16" t="s">
         <v>281</v>
-      </c>
-      <c r="B155" s="16" t="s">
-        <v>282</v>
       </c>
       <c r="C155" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D155" s="18"/>
       <c r="E155" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F155" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="G155" s="4" t="s">
         <v>283</v>
-      </c>
-      <c r="G155" s="4" t="s">
-        <v>284</v>
       </c>
       <c r="H155" s="19"/>
     </row>
     <row r="156" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="15" t="s">
+        <v>284</v>
+      </c>
+      <c r="B156" s="16" t="s">
         <v>285</v>
-      </c>
-      <c r="B156" s="16" t="s">
-        <v>286</v>
       </c>
       <c r="C156" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D156" s="18"/>
       <c r="E156" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F156" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="G156" s="4" t="s">
         <v>287</v>
-      </c>
-      <c r="G156" s="4" t="s">
-        <v>288</v>
       </c>
       <c r="H156" s="19"/>
     </row>
     <row r="157" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="B157" s="16" t="s">
         <v>289</v>
-      </c>
-      <c r="B157" s="16" t="s">
-        <v>290</v>
       </c>
       <c r="C157" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D157" s="18"/>
       <c r="E157" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F157" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="G157" s="4" t="s">
         <v>291</v>
-      </c>
-      <c r="G157" s="4" t="s">
-        <v>292</v>
       </c>
       <c r="H157" s="19"/>
     </row>
     <row r="158" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A158" s="15" t="s">
+        <v>292</v>
+      </c>
+      <c r="B158" s="16" t="s">
         <v>293</v>
-      </c>
-      <c r="B158" s="16" t="s">
-        <v>294</v>
       </c>
       <c r="C158" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D158" s="18"/>
       <c r="E158" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F158" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="G158" s="4" t="s">
         <v>295</v>
-      </c>
-      <c r="G158" s="4" t="s">
-        <v>296</v>
       </c>
       <c r="H158" s="19"/>
     </row>
     <row r="159" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="15" t="s">
+        <v>296</v>
+      </c>
+      <c r="B159" s="16" t="s">
         <v>297</v>
-      </c>
-      <c r="B159" s="16" t="s">
-        <v>298</v>
       </c>
       <c r="C159" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D159" s="18"/>
       <c r="E159" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F159" s="4" t="s">
         <v>113</v>
@@ -5400,10 +5400,10 @@
     </row>
     <row r="160" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="15" t="s">
+        <v>298</v>
+      </c>
+      <c r="B160" s="16" t="s">
         <v>299</v>
-      </c>
-      <c r="B160" s="16" t="s">
-        <v>300</v>
       </c>
       <c r="C160" s="22" t="s">
         <v>54</v>
@@ -5416,10 +5416,10 @@
     </row>
     <row r="161" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A161" s="15" t="s">
+        <v>300</v>
+      </c>
+      <c r="B161" s="16" t="s">
         <v>301</v>
-      </c>
-      <c r="B161" s="16" t="s">
-        <v>302</v>
       </c>
       <c r="C161" s="22" t="s">
         <v>44</v>
@@ -5432,10 +5432,10 @@
     </row>
     <row r="162" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" s="15" t="s">
+        <v>302</v>
+      </c>
+      <c r="B162" s="16" t="s">
         <v>303</v>
-      </c>
-      <c r="B162" s="16" t="s">
-        <v>304</v>
       </c>
       <c r="C162" s="22" t="s">
         <v>44</v>
@@ -5448,10 +5448,10 @@
     </row>
     <row r="163" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A163" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="B163" s="16" t="s">
         <v>305</v>
-      </c>
-      <c r="B163" s="16" t="s">
-        <v>306</v>
       </c>
       <c r="C163" s="22" t="s">
         <v>44</v>
@@ -5464,66 +5464,66 @@
     </row>
     <row r="164" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A164" s="25" t="s">
+        <v>306</v>
+      </c>
+      <c r="B164" s="16" t="s">
         <v>307</v>
-      </c>
-      <c r="B164" s="16" t="s">
-        <v>308</v>
       </c>
       <c r="C164" s="22" t="s">
         <v>54</v>
       </c>
       <c r="D164" s="24" t="s">
+        <v>308</v>
+      </c>
+      <c r="E164" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="F164" s="4" t="s">
         <v>309</v>
       </c>
-      <c r="E164" s="4" t="s">
-        <v>280</v>
-      </c>
-      <c r="F164" s="4" t="s">
+      <c r="G164" s="4" t="s">
         <v>310</v>
-      </c>
-      <c r="G164" s="4" t="s">
-        <v>311</v>
       </c>
       <c r="H164" s="19"/>
     </row>
     <row r="165" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A165" s="25" t="s">
+        <v>311</v>
+      </c>
+      <c r="B165" s="16" t="s">
         <v>312</v>
-      </c>
-      <c r="B165" s="16" t="s">
-        <v>313</v>
       </c>
       <c r="C165" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D165" s="18"/>
       <c r="E165" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F165" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="G165" s="4" t="s">
         <v>283</v>
-      </c>
-      <c r="G165" s="4" t="s">
-        <v>284</v>
       </c>
       <c r="H165" s="19"/>
     </row>
     <row r="166" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" s="25" t="s">
+        <v>313</v>
+      </c>
+      <c r="B166" s="16" t="s">
         <v>314</v>
-      </c>
-      <c r="B166" s="16" t="s">
-        <v>315</v>
       </c>
       <c r="C166" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D166" s="18"/>
       <c r="E166" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F166" s="4" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="G166" s="4" t="s">
         <v>114</v>
@@ -5532,46 +5532,46 @@
     </row>
     <row r="167" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A167" s="25" t="s">
+        <v>316</v>
+      </c>
+      <c r="B167" s="16" t="s">
         <v>317</v>
-      </c>
-      <c r="B167" s="16" t="s">
-        <v>318</v>
       </c>
       <c r="C167" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D167" s="18"/>
       <c r="E167" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F167" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="G167" s="4" t="s">
         <v>319</v>
-      </c>
-      <c r="G167" s="4" t="s">
-        <v>320</v>
       </c>
       <c r="H167" s="19"/>
     </row>
     <row r="168" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A168" s="25" t="s">
+        <v>320</v>
+      </c>
+      <c r="B168" s="16" t="s">
         <v>321</v>
-      </c>
-      <c r="B168" s="16" t="s">
-        <v>322</v>
       </c>
       <c r="C168" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D168" s="18"/>
       <c r="E168" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F168" s="4"/>
       <c r="G168" s="4"/>
       <c r="H168" s="19"/>
     </row>
     <row r="169" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A169" s="38"/>
+      <c r="A169" s="42"/>
       <c r="B169" s="39"/>
       <c r="C169" s="39"/>
       <c r="D169" s="39"/>
@@ -5582,7 +5582,7 @@
     </row>
     <row r="170" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A170" s="41" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B170" s="39"/>
       <c r="C170" s="39"/>
@@ -5593,8 +5593,8 @@
       <c r="H170" s="40"/>
     </row>
     <row r="171" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A171" s="47" t="s">
-        <v>324</v>
+      <c r="A171" s="38" t="s">
+        <v>323</v>
       </c>
       <c r="B171" s="39"/>
       <c r="C171" s="39"/>
@@ -5606,20 +5606,20 @@
     </row>
     <row r="172" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" s="25" t="s">
+        <v>324</v>
+      </c>
+      <c r="B172" s="34" t="s">
         <v>325</v>
-      </c>
-      <c r="B172" s="34" t="s">
-        <v>326</v>
       </c>
       <c r="C172" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D172" s="18"/>
       <c r="E172" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="F172" s="4" t="s">
         <v>327</v>
-      </c>
-      <c r="F172" s="4" t="s">
-        <v>328</v>
       </c>
       <c r="G172" s="4" t="s">
         <v>114</v>
@@ -5628,32 +5628,32 @@
     </row>
     <row r="173" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A173" s="25" t="s">
+        <v>328</v>
+      </c>
+      <c r="B173" s="16" t="s">
         <v>329</v>
-      </c>
-      <c r="B173" s="16" t="s">
-        <v>330</v>
       </c>
       <c r="C173" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D173" s="18"/>
       <c r="E173" s="4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="F173" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="G173" s="4" t="s">
         <v>331</v>
-      </c>
-      <c r="G173" s="4" t="s">
-        <v>332</v>
       </c>
       <c r="H173" s="19"/>
     </row>
     <row r="174" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" s="25" t="s">
+        <v>332</v>
+      </c>
+      <c r="B174" s="16" t="s">
         <v>333</v>
-      </c>
-      <c r="B174" s="16" t="s">
-        <v>334</v>
       </c>
       <c r="C174" s="22" t="s">
         <v>35</v>
@@ -5666,10 +5666,10 @@
     </row>
     <row r="175" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" s="25" t="s">
+        <v>334</v>
+      </c>
+      <c r="B175" s="16" t="s">
         <v>335</v>
-      </c>
-      <c r="B175" s="16" t="s">
-        <v>336</v>
       </c>
       <c r="C175" s="22" t="s">
         <v>35</v>
@@ -5681,7 +5681,7 @@
       <c r="H175" s="19"/>
     </row>
     <row r="176" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A176" s="38"/>
+      <c r="A176" s="42"/>
       <c r="B176" s="39"/>
       <c r="C176" s="39"/>
       <c r="D176" s="39"/>
@@ -5692,7 +5692,7 @@
     </row>
     <row r="177" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" s="41" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B177" s="39"/>
       <c r="C177" s="39"/>
@@ -5703,8 +5703,8 @@
       <c r="H177" s="40"/>
     </row>
     <row r="178" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A178" s="47" t="s">
-        <v>338</v>
+      <c r="A178" s="38" t="s">
+        <v>337</v>
       </c>
       <c r="B178" s="39"/>
       <c r="C178" s="39"/>
@@ -5716,10 +5716,10 @@
     </row>
     <row r="179" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" s="25" t="s">
+        <v>338</v>
+      </c>
+      <c r="B179" s="16" t="s">
         <v>339</v>
-      </c>
-      <c r="B179" s="16" t="s">
-        <v>340</v>
       </c>
       <c r="C179" s="22" t="s">
         <v>54</v>
@@ -5732,10 +5732,10 @@
     </row>
     <row r="180" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" s="25" t="s">
+        <v>340</v>
+      </c>
+      <c r="B180" s="16" t="s">
         <v>341</v>
-      </c>
-      <c r="B180" s="16" t="s">
-        <v>342</v>
       </c>
       <c r="C180" s="22" t="s">
         <v>35</v>
@@ -5748,10 +5748,10 @@
     </row>
     <row r="181" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" s="25" t="s">
+        <v>342</v>
+      </c>
+      <c r="B181" s="16" t="s">
         <v>343</v>
-      </c>
-      <c r="B181" s="16" t="s">
-        <v>344</v>
       </c>
       <c r="C181" s="22" t="s">
         <v>35</v>
@@ -5764,10 +5764,10 @@
     </row>
     <row r="182" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" s="25" t="s">
+        <v>344</v>
+      </c>
+      <c r="B182" s="16" t="s">
         <v>345</v>
-      </c>
-      <c r="B182" s="16" t="s">
-        <v>346</v>
       </c>
       <c r="C182" s="22" t="s">
         <v>35</v>
@@ -5780,10 +5780,10 @@
     </row>
     <row r="183" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A183" s="25" t="s">
+        <v>346</v>
+      </c>
+      <c r="B183" s="16" t="s">
         <v>347</v>
-      </c>
-      <c r="B183" s="16" t="s">
-        <v>348</v>
       </c>
       <c r="C183" s="22" t="s">
         <v>35</v>
@@ -5796,10 +5796,10 @@
     </row>
     <row r="184" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A184" s="25" t="s">
+        <v>348</v>
+      </c>
+      <c r="B184" s="16" t="s">
         <v>349</v>
-      </c>
-      <c r="B184" s="16" t="s">
-        <v>350</v>
       </c>
       <c r="C184" s="22" t="s">
         <v>35</v>
@@ -5812,10 +5812,10 @@
     </row>
     <row r="185" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A185" s="25" t="s">
+        <v>350</v>
+      </c>
+      <c r="B185" s="16" t="s">
         <v>351</v>
-      </c>
-      <c r="B185" s="16" t="s">
-        <v>352</v>
       </c>
       <c r="C185" s="22" t="s">
         <v>54</v>
@@ -5828,10 +5828,10 @@
     </row>
     <row r="186" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A186" s="25" t="s">
+        <v>352</v>
+      </c>
+      <c r="B186" s="16" t="s">
         <v>353</v>
-      </c>
-      <c r="B186" s="16" t="s">
-        <v>354</v>
       </c>
       <c r="C186" s="22" t="s">
         <v>35</v>
@@ -5844,10 +5844,10 @@
     </row>
     <row r="187" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A187" s="25" t="s">
+        <v>354</v>
+      </c>
+      <c r="B187" s="16" t="s">
         <v>355</v>
-      </c>
-      <c r="B187" s="16" t="s">
-        <v>356</v>
       </c>
       <c r="C187" s="22" t="s">
         <v>35</v>
@@ -5860,10 +5860,10 @@
     </row>
     <row r="188" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188" s="25" t="s">
+        <v>356</v>
+      </c>
+      <c r="B188" s="16" t="s">
         <v>357</v>
-      </c>
-      <c r="B188" s="16" t="s">
-        <v>358</v>
       </c>
       <c r="C188" s="22" t="s">
         <v>35</v>
@@ -5876,16 +5876,16 @@
     </row>
     <row r="189" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A189" s="25" t="s">
+        <v>358</v>
+      </c>
+      <c r="B189" s="16" t="s">
         <v>359</v>
-      </c>
-      <c r="B189" s="16" t="s">
-        <v>360</v>
       </c>
       <c r="C189" s="22" t="s">
         <v>54</v>
       </c>
       <c r="D189" s="24" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E189" s="4"/>
       <c r="F189" s="4"/>
@@ -5894,10 +5894,10 @@
     </row>
     <row r="190" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A190" s="25" t="s">
+        <v>361</v>
+      </c>
+      <c r="B190" s="16" t="s">
         <v>362</v>
-      </c>
-      <c r="B190" s="16" t="s">
-        <v>363</v>
       </c>
       <c r="C190" s="22" t="s">
         <v>44</v>
@@ -5910,10 +5910,10 @@
     </row>
     <row r="191" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A191" s="25" t="s">
+        <v>363</v>
+      </c>
+      <c r="B191" s="16" t="s">
         <v>364</v>
-      </c>
-      <c r="B191" s="16" t="s">
-        <v>365</v>
       </c>
       <c r="C191" s="22" t="s">
         <v>54</v>
@@ -5926,10 +5926,10 @@
     </row>
     <row r="192" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A192" s="25" t="s">
+        <v>365</v>
+      </c>
+      <c r="B192" s="16" t="s">
         <v>366</v>
-      </c>
-      <c r="B192" s="16" t="s">
-        <v>367</v>
       </c>
       <c r="C192" s="22" t="s">
         <v>35</v>
@@ -5942,10 +5942,10 @@
     </row>
     <row r="193" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A193" s="25" t="s">
+        <v>367</v>
+      </c>
+      <c r="B193" s="16" t="s">
         <v>368</v>
-      </c>
-      <c r="B193" s="16" t="s">
-        <v>369</v>
       </c>
       <c r="C193" s="22" t="s">
         <v>35</v>
@@ -5958,10 +5958,10 @@
     </row>
     <row r="194" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A194" s="25" t="s">
+        <v>369</v>
+      </c>
+      <c r="B194" s="16" t="s">
         <v>370</v>
-      </c>
-      <c r="B194" s="16" t="s">
-        <v>371</v>
       </c>
       <c r="C194" s="22" t="s">
         <v>35</v>
@@ -5974,10 +5974,10 @@
     </row>
     <row r="195" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A195" s="25" t="s">
+        <v>371</v>
+      </c>
+      <c r="B195" s="16" t="s">
         <v>372</v>
-      </c>
-      <c r="B195" s="16" t="s">
-        <v>373</v>
       </c>
       <c r="C195" s="22" t="s">
         <v>35</v>
@@ -5990,10 +5990,10 @@
     </row>
     <row r="196" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A196" s="25" t="s">
+        <v>373</v>
+      </c>
+      <c r="B196" s="16" t="s">
         <v>374</v>
-      </c>
-      <c r="B196" s="16" t="s">
-        <v>375</v>
       </c>
       <c r="C196" s="22" t="s">
         <v>35</v>
@@ -6006,10 +6006,10 @@
     </row>
     <row r="197" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A197" s="25" t="s">
+        <v>375</v>
+      </c>
+      <c r="B197" s="16" t="s">
         <v>376</v>
-      </c>
-      <c r="B197" s="16" t="s">
-        <v>377</v>
       </c>
       <c r="C197" s="22" t="s">
         <v>35</v>
@@ -6032,7 +6032,7 @@
     </row>
     <row r="199" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A199" s="41" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="B199" s="39"/>
       <c r="C199" s="39"/>
@@ -6043,8 +6043,8 @@
       <c r="H199" s="40"/>
     </row>
     <row r="200" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A200" s="47" t="s">
-        <v>379</v>
+      <c r="A200" s="38" t="s">
+        <v>378</v>
       </c>
       <c r="B200" s="39"/>
       <c r="C200" s="39"/>
@@ -6056,17 +6056,17 @@
     </row>
     <row r="201" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A201" s="25" t="s">
+        <v>379</v>
+      </c>
+      <c r="B201" s="16" t="s">
         <v>380</v>
-      </c>
-      <c r="B201" s="16" t="s">
-        <v>381</v>
       </c>
       <c r="C201" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D201" s="18"/>
       <c r="E201" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F201" s="4" t="s">
         <v>177</v>
@@ -6078,17 +6078,17 @@
     </row>
     <row r="202" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A202" s="15" t="s">
+        <v>382</v>
+      </c>
+      <c r="B202" s="16" t="s">
         <v>383</v>
-      </c>
-      <c r="B202" s="16" t="s">
-        <v>384</v>
       </c>
       <c r="C202" s="22" t="s">
         <v>44</v>
       </c>
       <c r="D202" s="18"/>
       <c r="E202" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F202" s="4" t="s">
         <v>177</v>
@@ -6100,20 +6100,20 @@
     </row>
     <row r="203" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A203" s="25" t="s">
+        <v>384</v>
+      </c>
+      <c r="B203" s="16" t="s">
         <v>385</v>
-      </c>
-      <c r="B203" s="16" t="s">
-        <v>386</v>
       </c>
       <c r="C203" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D203" s="18"/>
       <c r="E203" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F203" s="4" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="G203" s="4" t="s">
         <v>178</v>
@@ -6122,17 +6122,17 @@
     </row>
     <row r="204" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A204" s="25" t="s">
+        <v>387</v>
+      </c>
+      <c r="B204" s="16" t="s">
         <v>388</v>
-      </c>
-      <c r="B204" s="16" t="s">
-        <v>389</v>
       </c>
       <c r="C204" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D204" s="18"/>
       <c r="E204" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F204" s="4" t="s">
         <v>177</v>
@@ -6144,32 +6144,32 @@
     </row>
     <row r="205" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A205" s="25" t="s">
+        <v>389</v>
+      </c>
+      <c r="B205" s="16" t="s">
         <v>390</v>
-      </c>
-      <c r="B205" s="16" t="s">
-        <v>391</v>
       </c>
       <c r="C205" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D205" s="18"/>
       <c r="E205" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F205" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="G205" s="4" t="s">
         <v>392</v>
-      </c>
-      <c r="G205" s="4" t="s">
-        <v>393</v>
       </c>
       <c r="H205" s="19"/>
     </row>
     <row r="206" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A206" s="15" t="s">
+        <v>393</v>
+      </c>
+      <c r="B206" s="16" t="s">
         <v>394</v>
-      </c>
-      <c r="B206" s="16" t="s">
-        <v>395</v>
       </c>
       <c r="C206" s="22" t="s">
         <v>35</v>
@@ -6182,17 +6182,17 @@
     </row>
     <row r="207" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A207" s="25" t="s">
+        <v>395</v>
+      </c>
+      <c r="B207" s="16" t="s">
         <v>396</v>
-      </c>
-      <c r="B207" s="16" t="s">
-        <v>397</v>
       </c>
       <c r="C207" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D207" s="18"/>
       <c r="E207" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F207" s="4"/>
       <c r="G207" s="4"/>
@@ -6200,17 +6200,17 @@
     </row>
     <row r="208" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A208" s="25" t="s">
+        <v>397</v>
+      </c>
+      <c r="B208" s="16" t="s">
         <v>398</v>
-      </c>
-      <c r="B208" s="16" t="s">
-        <v>399</v>
       </c>
       <c r="C208" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D208" s="18"/>
       <c r="E208" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F208" s="4" t="s">
         <v>177</v>
@@ -6222,10 +6222,10 @@
     </row>
     <row r="209" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A209" s="25" t="s">
+        <v>399</v>
+      </c>
+      <c r="B209" s="16" t="s">
         <v>400</v>
-      </c>
-      <c r="B209" s="16" t="s">
-        <v>401</v>
       </c>
       <c r="C209" s="22" t="s">
         <v>35</v>
@@ -6238,10 +6238,10 @@
     </row>
     <row r="210" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A210" s="25" t="s">
+        <v>401</v>
+      </c>
+      <c r="B210" s="16" t="s">
         <v>402</v>
-      </c>
-      <c r="B210" s="16" t="s">
-        <v>403</v>
       </c>
       <c r="C210" s="22" t="s">
         <v>35</v>
@@ -6254,17 +6254,17 @@
     </row>
     <row r="211" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A211" s="25" t="s">
+        <v>403</v>
+      </c>
+      <c r="B211" s="16" t="s">
         <v>404</v>
-      </c>
-      <c r="B211" s="16" t="s">
-        <v>405</v>
       </c>
       <c r="C211" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D211" s="18"/>
       <c r="E211" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F211" s="4" t="s">
         <v>177</v>
@@ -6276,17 +6276,17 @@
     </row>
     <row r="212" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A212" s="25" t="s">
+        <v>405</v>
+      </c>
+      <c r="B212" s="16" t="s">
         <v>406</v>
-      </c>
-      <c r="B212" s="16" t="s">
-        <v>407</v>
       </c>
       <c r="C212" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D212" s="18"/>
       <c r="E212" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F212" s="4" t="s">
         <v>177</v>
@@ -6298,17 +6298,17 @@
     </row>
     <row r="213" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A213" s="25" t="s">
+        <v>407</v>
+      </c>
+      <c r="B213" s="16" t="s">
         <v>408</v>
-      </c>
-      <c r="B213" s="16" t="s">
-        <v>409</v>
       </c>
       <c r="C213" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D213" s="18"/>
       <c r="E213" s="4" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F213" s="4" t="s">
         <v>177</v>
@@ -6320,10 +6320,10 @@
     </row>
     <row r="214" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A214" s="25" t="s">
+        <v>409</v>
+      </c>
+      <c r="B214" s="16" t="s">
         <v>410</v>
-      </c>
-      <c r="B214" s="16" t="s">
-        <v>411</v>
       </c>
       <c r="C214" s="22" t="s">
         <v>35</v>
@@ -6336,10 +6336,10 @@
     </row>
     <row r="215" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A215" s="25" t="s">
+        <v>411</v>
+      </c>
+      <c r="B215" s="16" t="s">
         <v>412</v>
-      </c>
-      <c r="B215" s="16" t="s">
-        <v>413</v>
       </c>
       <c r="C215" s="22" t="s">
         <v>35</v>
@@ -6352,10 +6352,10 @@
     </row>
     <row r="216" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A216" s="25" t="s">
+        <v>413</v>
+      </c>
+      <c r="B216" s="16" t="s">
         <v>414</v>
-      </c>
-      <c r="B216" s="16" t="s">
-        <v>415</v>
       </c>
       <c r="C216" s="22" t="s">
         <v>35</v>
@@ -6368,10 +6368,10 @@
     </row>
     <row r="217" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A217" s="25" t="s">
+        <v>415</v>
+      </c>
+      <c r="B217" s="16" t="s">
         <v>416</v>
-      </c>
-      <c r="B217" s="16" t="s">
-        <v>417</v>
       </c>
       <c r="C217" s="22" t="s">
         <v>35</v>
@@ -6383,7 +6383,7 @@
       <c r="H217" s="19"/>
     </row>
     <row r="218" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A218" s="38"/>
+      <c r="A218" s="42"/>
       <c r="B218" s="39"/>
       <c r="C218" s="39"/>
       <c r="D218" s="39"/>
@@ -6394,7 +6394,7 @@
     </row>
     <row r="219" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A219" s="41" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="B219" s="39"/>
       <c r="C219" s="39"/>
@@ -6405,8 +6405,8 @@
       <c r="H219" s="40"/>
     </row>
     <row r="220" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A220" s="47" t="s">
-        <v>419</v>
+      <c r="A220" s="38" t="s">
+        <v>418</v>
       </c>
       <c r="B220" s="39"/>
       <c r="C220" s="39"/>
@@ -6418,94 +6418,94 @@
     </row>
     <row r="221" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A221" s="15" t="s">
+        <v>419</v>
+      </c>
+      <c r="B221" s="16" t="s">
         <v>420</v>
-      </c>
-      <c r="B221" s="16" t="s">
-        <v>421</v>
       </c>
       <c r="C221" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D221" s="18"/>
       <c r="E221" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="F221" s="4" t="s">
         <v>422</v>
       </c>
-      <c r="F221" s="4" t="s">
+      <c r="G221" s="4" t="s">
         <v>423</v>
-      </c>
-      <c r="G221" s="4" t="s">
-        <v>424</v>
       </c>
       <c r="H221" s="19"/>
     </row>
     <row r="222" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A222" s="15" t="s">
+        <v>424</v>
+      </c>
+      <c r="B222" s="16" t="s">
         <v>425</v>
-      </c>
-      <c r="B222" s="16" t="s">
-        <v>426</v>
       </c>
       <c r="C222" s="22" t="s">
         <v>54</v>
       </c>
       <c r="D222" s="18"/>
       <c r="E222" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="F222" s="4" t="s">
         <v>422</v>
       </c>
-      <c r="F222" s="4" t="s">
+      <c r="G222" s="4" t="s">
         <v>423</v>
-      </c>
-      <c r="G222" s="4" t="s">
-        <v>424</v>
       </c>
       <c r="H222" s="19"/>
     </row>
     <row r="223" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A223" s="15" t="s">
+        <v>426</v>
+      </c>
+      <c r="B223" s="16" t="s">
         <v>427</v>
-      </c>
-      <c r="B223" s="16" t="s">
-        <v>428</v>
       </c>
       <c r="C223" s="22" t="s">
         <v>54</v>
       </c>
       <c r="D223" s="18"/>
       <c r="E223" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="F223" s="4" t="s">
         <v>422</v>
       </c>
-      <c r="F223" s="4" t="s">
+      <c r="G223" s="4" t="s">
         <v>423</v>
-      </c>
-      <c r="G223" s="4" t="s">
-        <v>424</v>
       </c>
       <c r="H223" s="19"/>
     </row>
     <row r="224" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A224" s="15" t="s">
+        <v>428</v>
+      </c>
+      <c r="B224" s="16" t="s">
         <v>429</v>
-      </c>
-      <c r="B224" s="16" t="s">
-        <v>430</v>
       </c>
       <c r="C224" s="22" t="s">
         <v>44</v>
       </c>
       <c r="D224" s="18"/>
       <c r="E224" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="F224" s="4" t="s">
         <v>422</v>
       </c>
-      <c r="F224" s="4" t="s">
+      <c r="G224" s="4" t="s">
         <v>423</v>
       </c>
-      <c r="G224" s="4" t="s">
-        <v>424</v>
-      </c>
       <c r="H224" s="19"/>
     </row>
     <row r="225" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A225" s="38"/>
+      <c r="A225" s="42"/>
       <c r="B225" s="39"/>
       <c r="C225" s="39"/>
       <c r="D225" s="39"/>
@@ -6516,7 +6516,7 @@
     </row>
     <row r="226" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A226" s="41" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="B226" s="39"/>
       <c r="C226" s="39"/>
@@ -6527,8 +6527,8 @@
       <c r="H226" s="40"/>
     </row>
     <row r="227" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A227" s="47" t="s">
-        <v>432</v>
+      <c r="A227" s="38" t="s">
+        <v>431</v>
       </c>
       <c r="B227" s="39"/>
       <c r="C227" s="39"/>
@@ -6540,20 +6540,20 @@
     </row>
     <row r="228" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A228" s="15" t="s">
+        <v>432</v>
+      </c>
+      <c r="B228" s="16" t="s">
         <v>433</v>
-      </c>
-      <c r="B228" s="16" t="s">
-        <v>434</v>
       </c>
       <c r="C228" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D228" s="18"/>
       <c r="E228" s="4" t="s">
+        <v>434</v>
+      </c>
+      <c r="F228" s="4" t="s">
         <v>435</v>
-      </c>
-      <c r="F228" s="4" t="s">
-        <v>436</v>
       </c>
       <c r="G228" s="4" t="s">
         <v>114</v>
@@ -6562,74 +6562,74 @@
     </row>
     <row r="229" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A229" s="15" t="s">
+        <v>436</v>
+      </c>
+      <c r="B229" s="16" t="s">
         <v>437</v>
-      </c>
-      <c r="B229" s="16" t="s">
-        <v>438</v>
       </c>
       <c r="C229" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D229" s="18"/>
       <c r="E229" s="4" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="F229" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="G229" s="4" t="s">
         <v>439</v>
-      </c>
-      <c r="G229" s="4" t="s">
-        <v>440</v>
       </c>
       <c r="H229" s="19"/>
     </row>
     <row r="230" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A230" s="15" t="s">
+        <v>440</v>
+      </c>
+      <c r="B230" s="16" t="s">
         <v>441</v>
-      </c>
-      <c r="B230" s="16" t="s">
-        <v>442</v>
       </c>
       <c r="C230" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D230" s="24" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="E230" s="4" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="F230" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="G230" s="4" t="s">
         <v>439</v>
-      </c>
-      <c r="G230" s="4" t="s">
-        <v>440</v>
       </c>
       <c r="H230" s="19"/>
     </row>
     <row r="231" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A231" s="15" t="s">
+        <v>443</v>
+      </c>
+      <c r="B231" s="16" t="s">
         <v>444</v>
-      </c>
-      <c r="B231" s="16" t="s">
-        <v>445</v>
       </c>
       <c r="C231" s="22" t="s">
         <v>44</v>
       </c>
       <c r="D231" s="18"/>
       <c r="E231" s="4" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="F231" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="G231" s="4" t="s">
         <v>439</v>
       </c>
-      <c r="G231" s="4" t="s">
-        <v>440</v>
-      </c>
       <c r="H231" s="19"/>
     </row>
     <row r="232" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A232" s="48"/>
+      <c r="A232" s="47"/>
       <c r="B232" s="39"/>
       <c r="C232" s="39"/>
       <c r="D232" s="39"/>
@@ -6640,7 +6640,7 @@
     </row>
     <row r="233" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A233" s="41" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B233" s="39"/>
       <c r="C233" s="39"/>
@@ -6651,8 +6651,8 @@
       <c r="H233" s="40"/>
     </row>
     <row r="234" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A234" s="47" t="s">
-        <v>447</v>
+      <c r="A234" s="38" t="s">
+        <v>446</v>
       </c>
       <c r="B234" s="39"/>
       <c r="C234" s="39"/>
@@ -6664,10 +6664,10 @@
     </row>
     <row r="235" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A235" s="15" t="s">
+        <v>447</v>
+      </c>
+      <c r="B235" s="16" t="s">
         <v>448</v>
-      </c>
-      <c r="B235" s="16" t="s">
-        <v>449</v>
       </c>
       <c r="C235" s="22" t="s">
         <v>35</v>
@@ -6680,10 +6680,10 @@
     </row>
     <row r="236" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A236" s="15" t="s">
+        <v>449</v>
+      </c>
+      <c r="B236" s="16" t="s">
         <v>450</v>
-      </c>
-      <c r="B236" s="16" t="s">
-        <v>451</v>
       </c>
       <c r="C236" s="22" t="s">
         <v>35</v>
@@ -6696,10 +6696,10 @@
     </row>
     <row r="237" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A237" s="15" t="s">
+        <v>451</v>
+      </c>
+      <c r="B237" s="16" t="s">
         <v>452</v>
-      </c>
-      <c r="B237" s="16" t="s">
-        <v>453</v>
       </c>
       <c r="C237" s="22" t="s">
         <v>35</v>
@@ -6712,10 +6712,10 @@
     </row>
     <row r="238" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A238" s="15" t="s">
+        <v>453</v>
+      </c>
+      <c r="B238" s="16" t="s">
         <v>454</v>
-      </c>
-      <c r="B238" s="16" t="s">
-        <v>455</v>
       </c>
       <c r="C238" s="22" t="s">
         <v>35</v>
@@ -6728,10 +6728,10 @@
     </row>
     <row r="239" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A239" s="15" t="s">
+        <v>455</v>
+      </c>
+      <c r="B239" s="16" t="s">
         <v>456</v>
-      </c>
-      <c r="B239" s="16" t="s">
-        <v>457</v>
       </c>
       <c r="C239" s="22" t="s">
         <v>35</v>
@@ -6744,10 +6744,10 @@
     </row>
     <row r="240" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A240" s="15" t="s">
+        <v>457</v>
+      </c>
+      <c r="B240" s="16" t="s">
         <v>458</v>
-      </c>
-      <c r="B240" s="16" t="s">
-        <v>459</v>
       </c>
       <c r="C240" s="22" t="s">
         <v>35</v>
@@ -6760,10 +6760,10 @@
     </row>
     <row r="241" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A241" s="15" t="s">
+        <v>459</v>
+      </c>
+      <c r="B241" s="16" t="s">
         <v>460</v>
-      </c>
-      <c r="B241" s="16" t="s">
-        <v>461</v>
       </c>
       <c r="C241" s="22" t="s">
         <v>44</v>
@@ -6776,10 +6776,10 @@
     </row>
     <row r="242" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A242" s="15" t="s">
+        <v>461</v>
+      </c>
+      <c r="B242" s="16" t="s">
         <v>462</v>
-      </c>
-      <c r="B242" s="16" t="s">
-        <v>463</v>
       </c>
       <c r="C242" s="22" t="s">
         <v>44</v>
@@ -6792,10 +6792,10 @@
     </row>
     <row r="243" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A243" s="15" t="s">
+        <v>463</v>
+      </c>
+      <c r="B243" s="16" t="s">
         <v>464</v>
-      </c>
-      <c r="B243" s="16" t="s">
-        <v>465</v>
       </c>
       <c r="C243" s="22" t="s">
         <v>44</v>
@@ -6808,10 +6808,10 @@
     </row>
     <row r="244" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A244" s="15" t="s">
+        <v>465</v>
+      </c>
+      <c r="B244" s="16" t="s">
         <v>466</v>
-      </c>
-      <c r="B244" s="16" t="s">
-        <v>467</v>
       </c>
       <c r="C244" s="22" t="s">
         <v>44</v>
@@ -6824,10 +6824,10 @@
     </row>
     <row r="245" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A245" s="15" t="s">
+        <v>467</v>
+      </c>
+      <c r="B245" s="16" t="s">
         <v>468</v>
-      </c>
-      <c r="B245" s="16" t="s">
-        <v>469</v>
       </c>
       <c r="C245" s="22" t="s">
         <v>44</v>
@@ -6840,10 +6840,10 @@
     </row>
     <row r="246" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A246" s="15" t="s">
+        <v>469</v>
+      </c>
+      <c r="B246" s="16" t="s">
         <v>470</v>
-      </c>
-      <c r="B246" s="16" t="s">
-        <v>471</v>
       </c>
       <c r="C246" s="22" t="s">
         <v>35</v>
@@ -6856,10 +6856,10 @@
     </row>
     <row r="247" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A247" s="15" t="s">
+        <v>471</v>
+      </c>
+      <c r="B247" s="16" t="s">
         <v>472</v>
-      </c>
-      <c r="B247" s="16" t="s">
-        <v>473</v>
       </c>
       <c r="C247" s="22" t="s">
         <v>44</v>
@@ -6871,7 +6871,7 @@
       <c r="H247" s="19"/>
     </row>
     <row r="248" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A248" s="38"/>
+      <c r="A248" s="42"/>
       <c r="B248" s="39"/>
       <c r="C248" s="39"/>
       <c r="D248" s="39"/>
@@ -6882,7 +6882,7 @@
     </row>
     <row r="249" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A249" s="41" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B249" s="39"/>
       <c r="C249" s="39"/>
@@ -6893,8 +6893,8 @@
       <c r="H249" s="40"/>
     </row>
     <row r="250" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A250" s="47" t="s">
-        <v>475</v>
+      <c r="A250" s="38" t="s">
+        <v>474</v>
       </c>
       <c r="B250" s="39"/>
       <c r="C250" s="39"/>
@@ -6906,54 +6906,54 @@
     </row>
     <row r="251" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A251" s="15" t="s">
+        <v>475</v>
+      </c>
+      <c r="B251" s="16" t="s">
         <v>476</v>
-      </c>
-      <c r="B251" s="16" t="s">
-        <v>477</v>
       </c>
       <c r="C251" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D251" s="18"/>
       <c r="E251" s="4" t="s">
+        <v>477</v>
+      </c>
+      <c r="F251" s="4" t="s">
         <v>478</v>
       </c>
-      <c r="F251" s="4" t="s">
+      <c r="G251" s="4" t="s">
         <v>479</v>
-      </c>
-      <c r="G251" s="4" t="s">
-        <v>480</v>
       </c>
       <c r="H251" s="19"/>
     </row>
     <row r="252" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A252" s="15" t="s">
+        <v>480</v>
+      </c>
+      <c r="B252" s="16" t="s">
         <v>481</v>
-      </c>
-      <c r="B252" s="16" t="s">
-        <v>482</v>
       </c>
       <c r="C252" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D252" s="18"/>
       <c r="E252" s="4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F252" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="G252" s="4" t="s">
         <v>483</v>
-      </c>
-      <c r="G252" s="4" t="s">
-        <v>484</v>
       </c>
       <c r="H252" s="19"/>
     </row>
     <row r="253" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A253" s="15" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B253" s="34" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="C253" s="22" t="s">
         <v>35</v>
@@ -6966,10 +6966,10 @@
     </row>
     <row r="254" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A254" s="15" t="s">
+        <v>485</v>
+      </c>
+      <c r="B254" s="16" t="s">
         <v>486</v>
-      </c>
-      <c r="B254" s="16" t="s">
-        <v>487</v>
       </c>
       <c r="C254" s="22" t="s">
         <v>35</v>
@@ -6982,196 +6982,196 @@
     </row>
     <row r="255" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A255" s="15" t="s">
+        <v>487</v>
+      </c>
+      <c r="B255" s="16" t="s">
         <v>488</v>
-      </c>
-      <c r="B255" s="16" t="s">
-        <v>489</v>
       </c>
       <c r="C255" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D255" s="18"/>
       <c r="E255" s="4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F255" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="G255" s="4" t="s">
         <v>439</v>
-      </c>
-      <c r="G255" s="4" t="s">
-        <v>440</v>
       </c>
       <c r="H255" s="19"/>
     </row>
     <row r="256" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A256" s="15" t="s">
+        <v>489</v>
+      </c>
+      <c r="B256" s="16" t="s">
         <v>490</v>
-      </c>
-      <c r="B256" s="16" t="s">
-        <v>491</v>
       </c>
       <c r="C256" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D256" s="18"/>
       <c r="E256" s="4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F256" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="G256" s="4" t="s">
         <v>492</v>
-      </c>
-      <c r="G256" s="4" t="s">
-        <v>493</v>
       </c>
       <c r="H256" s="19"/>
     </row>
     <row r="257" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A257" s="15" t="s">
+        <v>493</v>
+      </c>
+      <c r="B257" s="16" t="s">
         <v>494</v>
-      </c>
-      <c r="B257" s="16" t="s">
-        <v>495</v>
       </c>
       <c r="C257" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D257" s="18"/>
       <c r="E257" s="4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F257" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G257" s="4" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="H257" s="19"/>
     </row>
     <row r="258" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A258" s="15" t="s">
+        <v>496</v>
+      </c>
+      <c r="B258" s="16" t="s">
         <v>497</v>
-      </c>
-      <c r="B258" s="16" t="s">
-        <v>498</v>
       </c>
       <c r="C258" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D258" s="18"/>
       <c r="E258" s="4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F258" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G258" s="4" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="H258" s="19"/>
     </row>
     <row r="259" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A259" s="15" t="s">
+        <v>498</v>
+      </c>
+      <c r="B259" s="16" t="s">
         <v>499</v>
-      </c>
-      <c r="B259" s="16" t="s">
-        <v>500</v>
       </c>
       <c r="C259" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D259" s="18"/>
       <c r="E259" s="4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F259" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="G259" s="4" t="s">
         <v>439</v>
-      </c>
-      <c r="G259" s="4" t="s">
-        <v>440</v>
       </c>
       <c r="H259" s="19"/>
     </row>
     <row r="260" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A260" s="15" t="s">
+        <v>500</v>
+      </c>
+      <c r="B260" s="16" t="s">
         <v>501</v>
-      </c>
-      <c r="B260" s="16" t="s">
-        <v>502</v>
       </c>
       <c r="C260" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D260" s="18"/>
       <c r="E260" s="4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F260" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G260" s="4" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="H260" s="19"/>
     </row>
     <row r="261" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A261" s="15" t="s">
+        <v>502</v>
+      </c>
+      <c r="B261" s="16" t="s">
         <v>503</v>
-      </c>
-      <c r="B261" s="16" t="s">
-        <v>504</v>
       </c>
       <c r="C261" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D261" s="18"/>
       <c r="E261" s="4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F261" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G261" s="4" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="H261" s="19"/>
     </row>
     <row r="262" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A262" s="15" t="s">
+        <v>504</v>
+      </c>
+      <c r="B262" s="16" t="s">
         <v>505</v>
-      </c>
-      <c r="B262" s="16" t="s">
-        <v>506</v>
       </c>
       <c r="C262" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D262" s="18"/>
       <c r="E262" s="4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F262" s="4" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G262" s="4" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="H262" s="19"/>
     </row>
     <row r="263" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A263" s="15" t="s">
+        <v>506</v>
+      </c>
+      <c r="B263" s="16" t="s">
         <v>507</v>
-      </c>
-      <c r="B263" s="16" t="s">
-        <v>508</v>
       </c>
       <c r="C263" s="22" t="s">
         <v>54</v>
       </c>
       <c r="D263" s="18"/>
       <c r="E263" s="4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F263" s="4" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="G263" s="4" t="s">
         <v>114</v>
@@ -7180,20 +7180,20 @@
     </row>
     <row r="264" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A264" s="15" t="s">
+        <v>509</v>
+      </c>
+      <c r="B264" s="16" t="s">
         <v>510</v>
-      </c>
-      <c r="B264" s="16" t="s">
-        <v>511</v>
       </c>
       <c r="C264" s="22" t="s">
         <v>54</v>
       </c>
       <c r="D264" s="18"/>
       <c r="E264" s="4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F264" s="4" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="G264" s="4" t="s">
         <v>114</v>
@@ -7202,32 +7202,32 @@
     </row>
     <row r="265" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A265" s="15" t="s">
+        <v>512</v>
+      </c>
+      <c r="B265" s="16" t="s">
         <v>513</v>
-      </c>
-      <c r="B265" s="16" t="s">
-        <v>514</v>
       </c>
       <c r="C265" s="22" t="s">
         <v>44</v>
       </c>
       <c r="D265" s="18"/>
       <c r="E265" s="4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F265" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="G265" s="4" t="s">
         <v>310</v>
-      </c>
-      <c r="G265" s="4" t="s">
-        <v>311</v>
       </c>
       <c r="H265" s="19"/>
     </row>
     <row r="266" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A266" s="15" t="s">
+        <v>514</v>
+      </c>
+      <c r="B266" s="16" t="s">
         <v>515</v>
-      </c>
-      <c r="B266" s="16" t="s">
-        <v>516</v>
       </c>
       <c r="C266" s="22" t="s">
         <v>54</v>
@@ -7240,10 +7240,10 @@
     </row>
     <row r="267" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A267" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B267" s="16" t="s">
         <v>517</v>
-      </c>
-      <c r="B267" s="16" t="s">
-        <v>518</v>
       </c>
       <c r="C267" s="22" t="s">
         <v>35</v>
@@ -7256,10 +7256,10 @@
     </row>
     <row r="268" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A268" s="15" t="s">
+        <v>518</v>
+      </c>
+      <c r="B268" s="16" t="s">
         <v>519</v>
-      </c>
-      <c r="B268" s="16" t="s">
-        <v>520</v>
       </c>
       <c r="C268" s="22" t="s">
         <v>35</v>
@@ -7272,10 +7272,10 @@
     </row>
     <row r="269" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A269" s="15" t="s">
+        <v>520</v>
+      </c>
+      <c r="B269" s="16" t="s">
         <v>521</v>
-      </c>
-      <c r="B269" s="16" t="s">
-        <v>522</v>
       </c>
       <c r="C269" s="22" t="s">
         <v>35</v>
@@ -7288,10 +7288,10 @@
     </row>
     <row r="270" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A270" s="15" t="s">
+        <v>522</v>
+      </c>
+      <c r="B270" s="16" t="s">
         <v>523</v>
-      </c>
-      <c r="B270" s="16" t="s">
-        <v>524</v>
       </c>
       <c r="C270" s="22" t="s">
         <v>35</v>
@@ -7304,10 +7304,10 @@
     </row>
     <row r="271" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A271" s="15" t="s">
+        <v>524</v>
+      </c>
+      <c r="B271" s="16" t="s">
         <v>525</v>
-      </c>
-      <c r="B271" s="16" t="s">
-        <v>526</v>
       </c>
       <c r="C271" s="22" t="s">
         <v>54</v>
@@ -7320,16 +7320,16 @@
     </row>
     <row r="272" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A272" s="15" t="s">
+        <v>526</v>
+      </c>
+      <c r="B272" s="36" t="s">
+        <v>628</v>
+      </c>
+      <c r="C272" s="35" t="s">
         <v>527</v>
       </c>
-      <c r="B272" s="36" t="s">
-        <v>629</v>
-      </c>
-      <c r="C272" s="35" t="s">
+      <c r="D272" s="36" t="s">
         <v>528</v>
-      </c>
-      <c r="D272" s="36" t="s">
-        <v>529</v>
       </c>
       <c r="E272" s="37"/>
       <c r="F272" s="37"/>
@@ -7337,7 +7337,7 @@
       <c r="H272" s="15"/>
     </row>
     <row r="273" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A273" s="51"/>
+      <c r="A273" s="52"/>
       <c r="B273" s="39"/>
       <c r="C273" s="39"/>
       <c r="D273" s="39"/>
@@ -7348,7 +7348,7 @@
     </row>
     <row r="274" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A274" s="41" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B274" s="39"/>
       <c r="C274" s="39"/>
@@ -7359,8 +7359,8 @@
       <c r="H274" s="40"/>
     </row>
     <row r="275" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A275" s="47" t="s">
-        <v>531</v>
+      <c r="A275" s="38" t="s">
+        <v>530</v>
       </c>
       <c r="B275" s="39"/>
       <c r="C275" s="39"/>
@@ -7372,78 +7372,78 @@
     </row>
     <row r="276" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A276" s="15" t="s">
+        <v>531</v>
+      </c>
+      <c r="B276" s="16" t="s">
         <v>532</v>
-      </c>
-      <c r="B276" s="16" t="s">
-        <v>533</v>
       </c>
       <c r="C276" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D276" s="18"/>
       <c r="E276" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="F276" s="4" t="s">
         <v>534</v>
       </c>
-      <c r="F276" s="4" t="s">
+      <c r="G276" s="4" t="s">
         <v>535</v>
-      </c>
-      <c r="G276" s="4" t="s">
-        <v>536</v>
       </c>
       <c r="H276" s="19"/>
     </row>
     <row r="277" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A277" s="15" t="s">
+        <v>536</v>
+      </c>
+      <c r="B277" s="16" t="s">
         <v>537</v>
-      </c>
-      <c r="B277" s="16" t="s">
-        <v>538</v>
       </c>
       <c r="C277" s="22" t="s">
         <v>54</v>
       </c>
       <c r="D277" s="24" t="s">
+        <v>538</v>
+      </c>
+      <c r="E277" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="F277" s="4" t="s">
         <v>539</v>
       </c>
-      <c r="E277" s="4" t="s">
-        <v>534</v>
-      </c>
-      <c r="F277" s="4" t="s">
+      <c r="G277" s="4" t="s">
         <v>540</v>
-      </c>
-      <c r="G277" s="4" t="s">
-        <v>541</v>
       </c>
       <c r="H277" s="19"/>
     </row>
     <row r="278" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A278" s="15" t="s">
+        <v>541</v>
+      </c>
+      <c r="B278" s="16" t="s">
         <v>542</v>
-      </c>
-      <c r="B278" s="16" t="s">
-        <v>543</v>
       </c>
       <c r="C278" s="22" t="s">
         <v>54</v>
       </c>
       <c r="D278" s="18"/>
       <c r="E278" s="4" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F278" s="4" t="s">
+        <v>543</v>
+      </c>
+      <c r="G278" s="4" t="s">
         <v>544</v>
-      </c>
-      <c r="G278" s="4" t="s">
-        <v>545</v>
       </c>
       <c r="H278" s="19"/>
     </row>
     <row r="279" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A279" s="15" t="s">
+        <v>545</v>
+      </c>
+      <c r="B279" s="16" t="s">
         <v>546</v>
-      </c>
-      <c r="B279" s="16" t="s">
-        <v>547</v>
       </c>
       <c r="C279" s="22" t="s">
         <v>44</v>
@@ -7456,10 +7456,10 @@
     </row>
     <row r="280" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A280" s="15" t="s">
+        <v>547</v>
+      </c>
+      <c r="B280" s="16" t="s">
         <v>548</v>
-      </c>
-      <c r="B280" s="16" t="s">
-        <v>549</v>
       </c>
       <c r="C280" s="22" t="s">
         <v>35</v>
@@ -7471,7 +7471,7 @@
       <c r="H280" s="19"/>
     </row>
     <row r="281" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A281" s="48"/>
+      <c r="A281" s="47"/>
       <c r="B281" s="39"/>
       <c r="C281" s="39"/>
       <c r="D281" s="39"/>
@@ -7482,7 +7482,7 @@
     </row>
     <row r="282" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A282" s="41" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B282" s="39"/>
       <c r="C282" s="39"/>
@@ -7493,8 +7493,8 @@
       <c r="H282" s="40"/>
     </row>
     <row r="283" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A283" s="47" t="s">
-        <v>551</v>
+      <c r="A283" s="38" t="s">
+        <v>550</v>
       </c>
       <c r="B283" s="39"/>
       <c r="C283" s="39"/>
@@ -7506,32 +7506,32 @@
     </row>
     <row r="284" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A284" s="15" t="s">
+        <v>551</v>
+      </c>
+      <c r="B284" s="16" t="s">
         <v>552</v>
-      </c>
-      <c r="B284" s="16" t="s">
-        <v>553</v>
       </c>
       <c r="C284" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D284" s="18"/>
       <c r="E284" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="F284" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="G284" s="4" t="s">
         <v>554</v>
-      </c>
-      <c r="F284" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="G284" s="4" t="s">
-        <v>555</v>
       </c>
       <c r="H284" s="19"/>
     </row>
     <row r="285" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A285" s="15" t="s">
+        <v>555</v>
+      </c>
+      <c r="B285" s="16" t="s">
         <v>556</v>
-      </c>
-      <c r="B285" s="16" t="s">
-        <v>557</v>
       </c>
       <c r="C285" s="22" t="s">
         <v>44</v>
@@ -7544,10 +7544,10 @@
     </row>
     <row r="286" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A286" s="15" t="s">
+        <v>557</v>
+      </c>
+      <c r="B286" s="16" t="s">
         <v>558</v>
-      </c>
-      <c r="B286" s="16" t="s">
-        <v>559</v>
       </c>
       <c r="C286" s="22" t="s">
         <v>44</v>
@@ -7560,10 +7560,10 @@
     </row>
     <row r="287" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A287" s="15" t="s">
+        <v>559</v>
+      </c>
+      <c r="B287" s="16" t="s">
         <v>560</v>
-      </c>
-      <c r="B287" s="16" t="s">
-        <v>561</v>
       </c>
       <c r="C287" s="22" t="s">
         <v>44</v>
@@ -7576,32 +7576,32 @@
     </row>
     <row r="288" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A288" s="15" t="s">
+        <v>561</v>
+      </c>
+      <c r="B288" s="16" t="s">
         <v>562</v>
-      </c>
-      <c r="B288" s="16" t="s">
-        <v>563</v>
       </c>
       <c r="C288" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D288" s="18"/>
       <c r="E288" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="F288" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="G288" s="4" t="s">
         <v>554</v>
-      </c>
-      <c r="F288" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="G288" s="4" t="s">
-        <v>555</v>
       </c>
       <c r="H288" s="19"/>
     </row>
     <row r="289" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A289" s="15" t="s">
+        <v>563</v>
+      </c>
+      <c r="B289" s="16" t="s">
         <v>564</v>
-      </c>
-      <c r="B289" s="16" t="s">
-        <v>565</v>
       </c>
       <c r="C289" s="22" t="s">
         <v>35</v>
@@ -7614,10 +7614,10 @@
     </row>
     <row r="290" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A290" s="15" t="s">
+        <v>565</v>
+      </c>
+      <c r="B290" s="16" t="s">
         <v>566</v>
-      </c>
-      <c r="B290" s="16" t="s">
-        <v>567</v>
       </c>
       <c r="C290" s="22" t="s">
         <v>35</v>
@@ -7629,7 +7629,7 @@
       <c r="H290" s="19"/>
     </row>
     <row r="291" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A291" s="38"/>
+      <c r="A291" s="42"/>
       <c r="B291" s="39"/>
       <c r="C291" s="39"/>
       <c r="D291" s="39"/>
@@ -7640,7 +7640,7 @@
     </row>
     <row r="292" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A292" s="41" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B292" s="39"/>
       <c r="C292" s="39"/>
@@ -7651,8 +7651,8 @@
       <c r="H292" s="40"/>
     </row>
     <row r="293" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A293" s="47" t="s">
-        <v>569</v>
+      <c r="A293" s="38" t="s">
+        <v>568</v>
       </c>
       <c r="B293" s="39"/>
       <c r="C293" s="39"/>
@@ -7664,54 +7664,54 @@
     </row>
     <row r="294" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A294" s="15" t="s">
+        <v>569</v>
+      </c>
+      <c r="B294" s="16" t="s">
         <v>570</v>
-      </c>
-      <c r="B294" s="16" t="s">
-        <v>571</v>
       </c>
       <c r="C294" s="22" t="s">
         <v>54</v>
       </c>
       <c r="D294" s="18"/>
       <c r="E294" s="4" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="F294" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="G294" s="4" t="s">
         <v>319</v>
-      </c>
-      <c r="G294" s="4" t="s">
-        <v>320</v>
       </c>
       <c r="H294" s="19"/>
     </row>
     <row r="295" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A295" s="15" t="s">
+        <v>572</v>
+      </c>
+      <c r="B295" s="16" t="s">
         <v>573</v>
-      </c>
-      <c r="B295" s="16" t="s">
-        <v>574</v>
       </c>
       <c r="C295" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D295" s="18"/>
       <c r="E295" s="4" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="F295" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="G295" s="4" t="s">
         <v>319</v>
-      </c>
-      <c r="G295" s="4" t="s">
-        <v>320</v>
       </c>
       <c r="H295" s="19"/>
     </row>
     <row r="296" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A296" s="15" t="s">
+        <v>574</v>
+      </c>
+      <c r="B296" s="16" t="s">
         <v>575</v>
-      </c>
-      <c r="B296" s="16" t="s">
-        <v>576</v>
       </c>
       <c r="C296" s="22" t="s">
         <v>35</v>
@@ -7724,54 +7724,54 @@
     </row>
     <row r="297" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A297" s="15" t="s">
+        <v>576</v>
+      </c>
+      <c r="B297" s="16" t="s">
         <v>577</v>
-      </c>
-      <c r="B297" s="16" t="s">
-        <v>578</v>
       </c>
       <c r="C297" s="22" t="s">
         <v>44</v>
       </c>
       <c r="D297" s="18"/>
       <c r="E297" s="4" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="F297" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="G297" s="4" t="s">
         <v>319</v>
-      </c>
-      <c r="G297" s="4" t="s">
-        <v>320</v>
       </c>
       <c r="H297" s="19"/>
     </row>
     <row r="298" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A298" s="15" t="s">
+        <v>578</v>
+      </c>
+      <c r="B298" s="16" t="s">
         <v>579</v>
-      </c>
-      <c r="B298" s="16" t="s">
-        <v>580</v>
       </c>
       <c r="C298" s="22" t="s">
         <v>44</v>
       </c>
       <c r="D298" s="18"/>
       <c r="E298" s="4" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="F298" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="G298" s="4" t="s">
         <v>319</v>
-      </c>
-      <c r="G298" s="4" t="s">
-        <v>320</v>
       </c>
       <c r="H298" s="19"/>
     </row>
     <row r="299" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A299" s="15" t="s">
+        <v>580</v>
+      </c>
+      <c r="B299" s="16" t="s">
         <v>581</v>
-      </c>
-      <c r="B299" s="16" t="s">
-        <v>582</v>
       </c>
       <c r="C299" s="22" t="s">
         <v>35</v>
@@ -7783,7 +7783,7 @@
       <c r="H299" s="19"/>
     </row>
     <row r="300" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A300" s="38"/>
+      <c r="A300" s="42"/>
       <c r="B300" s="39"/>
       <c r="C300" s="39"/>
       <c r="D300" s="39"/>
@@ -7794,7 +7794,7 @@
     </row>
     <row r="301" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A301" s="41" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B301" s="39"/>
       <c r="C301" s="39"/>
@@ -7805,8 +7805,8 @@
       <c r="H301" s="40"/>
     </row>
     <row r="302" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A302" s="47" t="s">
-        <v>584</v>
+      <c r="A302" s="38" t="s">
+        <v>583</v>
       </c>
       <c r="B302" s="39"/>
       <c r="C302" s="39"/>
@@ -7818,32 +7818,32 @@
     </row>
     <row r="303" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A303" s="15" t="s">
+        <v>584</v>
+      </c>
+      <c r="B303" s="16" t="s">
         <v>585</v>
-      </c>
-      <c r="B303" s="16" t="s">
-        <v>586</v>
       </c>
       <c r="C303" s="22" t="s">
         <v>35</v>
       </c>
       <c r="D303" s="18"/>
       <c r="E303" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F303" s="4" t="s">
         <v>587</v>
       </c>
-      <c r="F303" s="4" t="s">
+      <c r="G303" s="4" t="s">
         <v>588</v>
-      </c>
-      <c r="G303" s="4" t="s">
-        <v>589</v>
       </c>
       <c r="H303" s="19"/>
     </row>
     <row r="304" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A304" s="15" t="s">
+        <v>589</v>
+      </c>
+      <c r="B304" s="16" t="s">
         <v>590</v>
-      </c>
-      <c r="B304" s="16" t="s">
-        <v>591</v>
       </c>
       <c r="C304" s="22" t="s">
         <v>35</v>
@@ -7855,7 +7855,7 @@
       <c r="H304" s="19"/>
     </row>
     <row r="305" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A305" s="48"/>
+      <c r="A305" s="47"/>
       <c r="B305" s="39"/>
       <c r="C305" s="39"/>
       <c r="D305" s="39"/>
@@ -7866,7 +7866,7 @@
     </row>
     <row r="306" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A306" s="41" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B306" s="39"/>
       <c r="C306" s="39"/>
@@ -7877,8 +7877,8 @@
       <c r="H306" s="40"/>
     </row>
     <row r="307" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A307" s="47" t="s">
-        <v>593</v>
+      <c r="A307" s="38" t="s">
+        <v>592</v>
       </c>
       <c r="B307" s="39"/>
       <c r="C307" s="39"/>
@@ -7890,10 +7890,10 @@
     </row>
     <row r="308" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A308" s="15" t="s">
+        <v>593</v>
+      </c>
+      <c r="B308" s="16" t="s">
         <v>594</v>
-      </c>
-      <c r="B308" s="16" t="s">
-        <v>595</v>
       </c>
       <c r="C308" s="22" t="s">
         <v>35</v>
@@ -7901,19 +7901,19 @@
       <c r="D308" s="18"/>
       <c r="E308" s="26"/>
       <c r="F308" s="27" t="s">
+        <v>595</v>
+      </c>
+      <c r="G308" s="28" t="s">
         <v>596</v>
-      </c>
-      <c r="G308" s="28" t="s">
-        <v>597</v>
       </c>
       <c r="H308" s="19"/>
     </row>
     <row r="309" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A309" s="15" t="s">
+        <v>597</v>
+      </c>
+      <c r="B309" s="16" t="s">
         <v>598</v>
-      </c>
-      <c r="B309" s="16" t="s">
-        <v>599</v>
       </c>
       <c r="C309" s="22" t="s">
         <v>44</v>
@@ -7926,10 +7926,10 @@
     </row>
     <row r="310" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A310" s="15" t="s">
+        <v>599</v>
+      </c>
+      <c r="B310" s="16" t="s">
         <v>600</v>
-      </c>
-      <c r="B310" s="16" t="s">
-        <v>601</v>
       </c>
       <c r="C310" s="22" t="s">
         <v>44</v>
@@ -7942,10 +7942,10 @@
     </row>
     <row r="311" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A311" s="15" t="s">
+        <v>601</v>
+      </c>
+      <c r="B311" s="16" t="s">
         <v>602</v>
-      </c>
-      <c r="B311" s="16" t="s">
-        <v>603</v>
       </c>
       <c r="C311" s="22" t="s">
         <v>44</v>
@@ -7953,19 +7953,19 @@
       <c r="D311" s="18"/>
       <c r="E311" s="26"/>
       <c r="F311" s="27" t="s">
+        <v>595</v>
+      </c>
+      <c r="G311" s="28" t="s">
         <v>596</v>
-      </c>
-      <c r="G311" s="28" t="s">
-        <v>597</v>
       </c>
       <c r="H311" s="19"/>
     </row>
     <row r="312" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A312" s="15" t="s">
+        <v>603</v>
+      </c>
+      <c r="B312" s="16" t="s">
         <v>604</v>
-      </c>
-      <c r="B312" s="16" t="s">
-        <v>605</v>
       </c>
       <c r="C312" s="22" t="s">
         <v>44</v>
@@ -7978,10 +7978,10 @@
     </row>
     <row r="313" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A313" s="15" t="s">
+        <v>605</v>
+      </c>
+      <c r="B313" s="16" t="s">
         <v>606</v>
-      </c>
-      <c r="B313" s="16" t="s">
-        <v>607</v>
       </c>
       <c r="C313" s="22" t="s">
         <v>44</v>
@@ -7993,7 +7993,7 @@
       <c r="H313" s="19"/>
     </row>
     <row r="314" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A314" s="48"/>
+      <c r="A314" s="47"/>
       <c r="B314" s="39"/>
       <c r="C314" s="39"/>
       <c r="D314" s="39"/>
@@ -8004,7 +8004,7 @@
     </row>
     <row r="315" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A315" s="41" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B315" s="39"/>
       <c r="C315" s="39"/>
@@ -8017,7 +8017,7 @@
     <row r="316" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A316" s="29"/>
       <c r="B316" s="30" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="C316" s="31"/>
       <c r="D316" s="31"/>
@@ -8027,8 +8027,8 @@
       <c r="H316" s="19"/>
     </row>
     <row r="317" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A317" s="48" t="s">
-        <v>610</v>
+      <c r="A317" s="47" t="s">
+        <v>609</v>
       </c>
       <c r="B317" s="39"/>
       <c r="C317" s="39"/>
@@ -8040,7 +8040,7 @@
     </row>
     <row r="318" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A318" s="41" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B318" s="39"/>
       <c r="C318" s="39"/>
@@ -8052,101 +8052,101 @@
     </row>
     <row r="319" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A319" s="15" t="s">
+        <v>611</v>
+      </c>
+      <c r="B319" s="50" t="s">
         <v>612</v>
-      </c>
-      <c r="B319" s="42" t="s">
-        <v>613</v>
       </c>
       <c r="C319" s="39"/>
       <c r="D319" s="40"/>
       <c r="E319" s="4"/>
       <c r="F319" s="4"/>
       <c r="G319" s="4"/>
-      <c r="H319" s="44"/>
+      <c r="H319" s="54"/>
     </row>
     <row r="320" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A320" s="15" t="s">
+        <v>613</v>
+      </c>
+      <c r="B320" s="50" t="s">
         <v>614</v>
-      </c>
-      <c r="B320" s="42" t="s">
-        <v>615</v>
       </c>
       <c r="C320" s="39"/>
       <c r="D320" s="40"/>
       <c r="E320" s="4"/>
       <c r="F320" s="4"/>
       <c r="G320" s="4"/>
-      <c r="H320" s="45"/>
+      <c r="H320" s="55"/>
     </row>
     <row r="321" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A321" s="15" t="s">
+        <v>615</v>
+      </c>
+      <c r="B321" s="50" t="s">
         <v>616</v>
-      </c>
-      <c r="B321" s="42" t="s">
-        <v>617</v>
       </c>
       <c r="C321" s="39"/>
       <c r="D321" s="40"/>
       <c r="E321" s="4"/>
       <c r="F321" s="4"/>
       <c r="G321" s="4"/>
-      <c r="H321" s="45"/>
+      <c r="H321" s="55"/>
     </row>
     <row r="322" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A322" s="15" t="s">
+        <v>617</v>
+      </c>
+      <c r="B322" s="50" t="s">
         <v>618</v>
-      </c>
-      <c r="B322" s="42" t="s">
-        <v>619</v>
       </c>
       <c r="C322" s="39"/>
       <c r="D322" s="40"/>
       <c r="E322" s="4"/>
       <c r="F322" s="4"/>
       <c r="G322" s="4"/>
-      <c r="H322" s="45"/>
+      <c r="H322" s="55"/>
     </row>
     <row r="323" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A323" s="15" t="s">
+        <v>619</v>
+      </c>
+      <c r="B323" s="51" t="s">
         <v>620</v>
-      </c>
-      <c r="B323" s="50" t="s">
-        <v>621</v>
       </c>
       <c r="C323" s="39"/>
       <c r="D323" s="40"/>
       <c r="E323" s="4"/>
       <c r="F323" s="4"/>
       <c r="G323" s="4"/>
-      <c r="H323" s="45"/>
+      <c r="H323" s="55"/>
     </row>
     <row r="324" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A324" s="15" t="s">
+        <v>621</v>
+      </c>
+      <c r="B324" s="50" t="s">
         <v>622</v>
-      </c>
-      <c r="B324" s="42" t="s">
-        <v>623</v>
       </c>
       <c r="C324" s="39"/>
       <c r="D324" s="40"/>
       <c r="E324" s="4"/>
       <c r="F324" s="4"/>
       <c r="G324" s="4"/>
-      <c r="H324" s="45"/>
+      <c r="H324" s="55"/>
     </row>
     <row r="325" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A325" s="15" t="s">
+        <v>623</v>
+      </c>
+      <c r="B325" s="53" t="s">
         <v>624</v>
-      </c>
-      <c r="B325" s="43" t="s">
-        <v>625</v>
       </c>
       <c r="C325" s="39"/>
       <c r="D325" s="40"/>
       <c r="E325" s="4"/>
       <c r="F325" s="4"/>
       <c r="G325" s="4"/>
-      <c r="H325" s="46"/>
+      <c r="H325" s="56"/>
     </row>
     <row r="326" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B326" s="32"/>
@@ -13326,18 +13326,57 @@
     </row>
   </sheetData>
   <mergeCells count="79">
-    <mergeCell ref="A50:H50"/>
-    <mergeCell ref="A53:H53"/>
-    <mergeCell ref="A52:H52"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A24:H24"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A48:H48"/>
-    <mergeCell ref="A49:H49"/>
+    <mergeCell ref="A300:H300"/>
+    <mergeCell ref="A301:H301"/>
+    <mergeCell ref="B319:D319"/>
+    <mergeCell ref="B320:D320"/>
+    <mergeCell ref="B324:D324"/>
+    <mergeCell ref="B325:D325"/>
+    <mergeCell ref="H319:H325"/>
+    <mergeCell ref="A302:H302"/>
+    <mergeCell ref="A305:H305"/>
+    <mergeCell ref="A306:H306"/>
+    <mergeCell ref="A307:H307"/>
+    <mergeCell ref="A314:H314"/>
+    <mergeCell ref="A315:H315"/>
+    <mergeCell ref="A318:H318"/>
+    <mergeCell ref="A317:H317"/>
+    <mergeCell ref="A138:H138"/>
+    <mergeCell ref="A198:H198"/>
+    <mergeCell ref="B321:D321"/>
+    <mergeCell ref="B322:D322"/>
+    <mergeCell ref="B323:D323"/>
+    <mergeCell ref="A249:H249"/>
+    <mergeCell ref="A250:H250"/>
+    <mergeCell ref="A273:H273"/>
+    <mergeCell ref="A274:H274"/>
+    <mergeCell ref="A275:H275"/>
+    <mergeCell ref="A281:H281"/>
+    <mergeCell ref="A282:H282"/>
+    <mergeCell ref="A283:H283"/>
+    <mergeCell ref="A291:H291"/>
+    <mergeCell ref="A292:H292"/>
+    <mergeCell ref="A293:H293"/>
+    <mergeCell ref="A132:H132"/>
+    <mergeCell ref="A133:H133"/>
+    <mergeCell ref="A134:H134"/>
+    <mergeCell ref="A136:H136"/>
+    <mergeCell ref="A137:H137"/>
+    <mergeCell ref="A88:H88"/>
+    <mergeCell ref="A89:H89"/>
+    <mergeCell ref="A95:H95"/>
+    <mergeCell ref="A96:H96"/>
+    <mergeCell ref="A97:H97"/>
+    <mergeCell ref="A227:H227"/>
+    <mergeCell ref="A232:H232"/>
+    <mergeCell ref="A233:H233"/>
+    <mergeCell ref="A234:H234"/>
+    <mergeCell ref="A248:H248"/>
+    <mergeCell ref="A218:H218"/>
+    <mergeCell ref="A219:H219"/>
+    <mergeCell ref="A220:H220"/>
+    <mergeCell ref="A225:H225"/>
+    <mergeCell ref="A226:H226"/>
     <mergeCell ref="A54:H54"/>
     <mergeCell ref="A199:H199"/>
     <mergeCell ref="A200:H200"/>
@@ -13354,57 +13393,18 @@
     <mergeCell ref="A151:H151"/>
     <mergeCell ref="A153:H153"/>
     <mergeCell ref="A87:H87"/>
-    <mergeCell ref="A218:H218"/>
-    <mergeCell ref="A219:H219"/>
-    <mergeCell ref="A220:H220"/>
-    <mergeCell ref="A225:H225"/>
-    <mergeCell ref="A226:H226"/>
-    <mergeCell ref="A227:H227"/>
-    <mergeCell ref="A232:H232"/>
-    <mergeCell ref="A233:H233"/>
-    <mergeCell ref="A234:H234"/>
-    <mergeCell ref="A248:H248"/>
-    <mergeCell ref="A88:H88"/>
-    <mergeCell ref="A89:H89"/>
-    <mergeCell ref="A95:H95"/>
-    <mergeCell ref="A96:H96"/>
-    <mergeCell ref="A97:H97"/>
-    <mergeCell ref="A132:H132"/>
-    <mergeCell ref="A133:H133"/>
-    <mergeCell ref="A134:H134"/>
-    <mergeCell ref="A136:H136"/>
-    <mergeCell ref="A137:H137"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="A198:H198"/>
-    <mergeCell ref="B321:D321"/>
-    <mergeCell ref="B322:D322"/>
-    <mergeCell ref="B323:D323"/>
-    <mergeCell ref="A249:H249"/>
-    <mergeCell ref="A250:H250"/>
-    <mergeCell ref="A273:H273"/>
-    <mergeCell ref="A274:H274"/>
-    <mergeCell ref="A275:H275"/>
-    <mergeCell ref="A281:H281"/>
-    <mergeCell ref="A282:H282"/>
-    <mergeCell ref="A283:H283"/>
-    <mergeCell ref="A291:H291"/>
-    <mergeCell ref="A292:H292"/>
-    <mergeCell ref="A293:H293"/>
-    <mergeCell ref="B325:D325"/>
-    <mergeCell ref="H319:H325"/>
-    <mergeCell ref="A302:H302"/>
-    <mergeCell ref="A305:H305"/>
-    <mergeCell ref="A306:H306"/>
-    <mergeCell ref="A307:H307"/>
-    <mergeCell ref="A314:H314"/>
-    <mergeCell ref="A315:H315"/>
-    <mergeCell ref="A318:H318"/>
-    <mergeCell ref="A317:H317"/>
-    <mergeCell ref="A300:H300"/>
-    <mergeCell ref="A301:H301"/>
-    <mergeCell ref="B319:D319"/>
-    <mergeCell ref="B320:D320"/>
-    <mergeCell ref="B324:D324"/>
+    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="A53:H53"/>
+    <mergeCell ref="A52:H52"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A48:H48"/>
+    <mergeCell ref="A49:H49"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C16:C23 C26:C47 C51 C55:C58 C60:C61 C63:C86 C90:C94 C98:C131 C135 C139:C145 C149:C150 C154:C168 C172:C175 C179:C197 C201:C217 C221:C224 C228:C231 C235:C247 C251:C272 C276:C280 C284:C290 C294:C299 C303:C304 C308:C313" xr:uid="{00000000-0002-0000-0000-000000000000}">

</xml_diff>